<commit_message>
docs: update weekly progress, frontend work log and project timeline
</commit_message>
<xml_diff>
--- a/reports/09-timeline/Project_Timeline.xlsx
+++ b/reports/09-timeline/Project_Timeline.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="150">
   <si>
     <t xml:space="preserve">POS System: 10-week project timeline</t>
   </si>
@@ -79,69 +79,69 @@
     <t xml:space="preserve">13dc390, 4584088, 80c721c, ef6144e, ddf392b, 751e82d</t>
   </si>
   <si>
-    <t xml:space="preserve">Design, SRS and Redux split</t>
+    <t xml:space="preserve">Design and Redux split</t>
   </si>
   <si>
     <t xml:space="preserve">Vrushay, Subhash</t>
   </si>
   <si>
-    <t xml:space="preserve">UML and ER diagrams (done), SRS in IEEE format, Redux Toolkit split: part 1 by Vrushay (done), part 2 and globleState.js by Subhash.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS, Design, Implementation</t>
+    <t xml:space="preserve">UML and ER diagrams, Redux Toolkit split: part 1 by Vrushay, part 2 and globleState.js by Subhash.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design, Implementation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11645a2, dbcae3a, 7ab1196 to 9809d35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin and onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subhash, Vrushay, Tanya (onboarding)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin pages: dashboard, stores, store details, pending requests, subscription plans, settings. Login, forgot password and onboarding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7307504 (onboarding owner details)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store pages (11): dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager and Cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishvas (Branch Manager), Vimal (Cashier)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager pages (9) and Cashier pages (5): POS screen, returns, order history, customer lookup, shift summary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3197520, bb95311, db9c60b, 3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vrushay with the whole team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postman report and 96-case sheet done. Run the collection with all role tokens, record results, negative and security tests, bug fixes.</t>
   </si>
   <si>
     <t xml:space="preserve">In progress</t>
   </si>
   <si>
-    <t xml:space="preserve">11645a2, dbcae3a, 7ab1196 to 9809d35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin and onboarding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subhash, Vrushay, Tanya (onboarding)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin pages: dashboard, stores, store details, pending requests, subscription plans, settings. Login, forgot password and onboarding.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7307504 (onboarding owner details)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tanya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store pages (11): dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager and Cashier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vishvas (Branch Manager), Vimal (Cashier)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager pages (9) and Cashier pages (5): POS screen, returns, order history, customer lookup, shift summary.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3197520, bb95311, db9c60b, 3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vrushay with the whole team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run the Postman collection with all role tokens, record results in the 96-case sheet, negative and security tests, bug fixes.</t>
-  </si>
-  <si>
     <t xml:space="preserve">9e2ca1a, 8172cb7 (report), test case sheet</t>
   </si>
   <si>
@@ -157,10 +157,10 @@
     <t xml:space="preserve">Planned</t>
   </si>
   <si>
-    <t xml:space="preserve">Code quality and documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axios interceptor, logout fix, API URL in env file, remove console logs, fix security findings, update README.</t>
+    <t xml:space="preserve">Code quality, SRS and documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS in IEEE format, Axios interceptor, logout fix, API URL in env file, remove console logs, fix security findings, update README.</t>
   </si>
   <si>
     <t xml:space="preserve">Implementation &amp; Code Quality</t>
@@ -220,9 +220,6 @@
     <t xml:space="preserve">dbcae3a, 7ab1196, 0abb5fc, 06b282a, 09a4708, 26e7b01, 8d7cd95, b04b449, ed775da, e426064, c579b5a, 9809d35</t>
   </si>
   <si>
-    <t xml:space="preserve">Part 1 done, Super Admin in progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">Subhash Dhaka</t>
   </si>
   <si>
@@ -238,9 +235,6 @@
     <t xml:space="preserve">ddf392b, 751e82d</t>
   </si>
   <si>
-    <t xml:space="preserve">Folder structure done, rest in progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vimal Kumar</t>
   </si>
   <si>
@@ -409,24 +403,21 @@
     <t xml:space="preserve">Super Admin module (Subhash and Vrushay)</t>
   </si>
   <si>
-    <t xml:space="preserve">commits going to the team repo</t>
+    <t xml:space="preserve">commits in the team repo</t>
   </si>
   <si>
     <t xml:space="preserve">Redux Toolkit part 2 and globleState.js (Subhash)</t>
   </si>
   <si>
-    <t xml:space="preserve">not pushed yet</t>
+    <t xml:space="preserve">Run the Postman collection and record results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test case sheet</t>
   </si>
   <si>
     <t xml:space="preserve">Pending</t>
   </si>
   <si>
-    <t xml:space="preserve">Run the Postman collection and record results</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test case sheet</t>
-  </si>
-  <si>
     <t xml:space="preserve">Progress by marks component</t>
   </si>
   <si>
@@ -463,7 +454,7 @@
     <t xml:space="preserve">Commit log, frontend work log, timeline and weekly reports. Update every week.</t>
   </si>
   <si>
-    <t xml:space="preserve">Backend and Redux part 1 done. Frontend modules in progress.</t>
+    <t xml:space="preserve">Backend, Redux Toolkit and all frontend modules done. Code quality fixes pending.</t>
   </si>
   <si>
     <t xml:space="preserve">Report and 96 test cases written, results to be recorded.</t>
@@ -1060,10 +1051,10 @@
         <v>21</v>
       </c>
       <c r="H7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1079,22 +1070,22 @@
         <v>46229</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1110,19 +1101,19 @@
         <v>46236</v>
       </c>
       <c r="D9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>31</v>
-      </c>
       <c r="G9" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I9" s="9"/>
     </row>
@@ -1139,22 +1130,22 @@
         <v>46243</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1170,19 +1161,19 @@
         <v>46250</v>
       </c>
       <c r="D11" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>22</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>39</v>
@@ -1210,7 +1201,7 @@
         <v>42</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>43</v>
@@ -1310,16 +1301,16 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"Done")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"In progress")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1405,92 +1396,92 @@
         <v>64</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="C5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>70</v>
-      </c>
       <c r="F5" s="9" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="F6" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="D7" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="F7" s="9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>86</v>
-      </c>
       <c r="F8" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D10" s="12" t="n">
         <f aca="false">6+5+9+11</f>
@@ -1499,7 +1490,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1531,15 +1522,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>9</v>
@@ -1559,16 +1550,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>16</v>
@@ -1579,16 +1570,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>16</v>
@@ -1599,16 +1590,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>16</v>
@@ -1619,16 +1610,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>16</v>
@@ -1639,16 +1630,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>16</v>
@@ -1659,16 +1650,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>16</v>
@@ -1679,16 +1670,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>16</v>
@@ -1699,16 +1690,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>16</v>
@@ -1719,16 +1710,16 @@
         <v>9</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>16</v>
@@ -1739,16 +1730,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>16</v>
@@ -1759,16 +1750,16 @@
         <v>11</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>16</v>
@@ -1779,16 +1770,16 @@
         <v>12</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>16</v>
@@ -1799,16 +1790,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>16</v>
@@ -1819,19 +1810,19 @@
         <v>14</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1839,19 +1830,19 @@
         <v>15</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1859,19 +1850,19 @@
         <v>16</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1879,19 +1870,19 @@
         <v>17</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20" s="6" t="n">
         <v>4</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1899,19 +1890,19 @@
         <v>18</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>3</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1919,19 +1910,19 @@
         <v>19</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D22" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>131</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1939,19 +1930,19 @@
         <v>20</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1960,12 +1951,12 @@
       </c>
       <c r="C25" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"Done")</f>
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C26" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"Made, not committed")</f>
@@ -1974,20 +1965,20 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"In progress")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"Pending")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2017,26 +2008,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>5</v>
@@ -2045,26 +2036,26 @@
         <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>10</v>
@@ -2073,24 +2064,24 @@
         <v>16</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>25</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>46</v>
       </c>
@@ -2098,53 +2089,53 @@
         <v>20</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C9" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>10</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D11" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">SUM(B4:B11)</f>
@@ -2153,7 +2144,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">SUMIF(C4:C11,"&lt;&gt;Not started",B4:B11)</f>
@@ -2162,7 +2153,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">B14/B13</f>

</xml_diff>

<commit_message>
docs(timeline): update the timeline with real commit counts and module owners
</commit_message>
<xml_diff>
--- a/reports/09-timeline/Project_Timeline.xlsx
+++ b/reports/09-timeline/Project_Timeline.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="164">
   <si>
     <t xml:space="preserve">POS System: 10-week project timeline</t>
   </si>
@@ -85,19 +85,22 @@
     <t xml:space="preserve">Vrushay, Subhash</t>
   </si>
   <si>
-    <t xml:space="preserve">UML and ER diagrams, Redux Toolkit split: part 1 by Vrushay, part 2 and globleState.js by Subhash.</t>
+    <t xml:space="preserve">UML and ER diagrams (done), Redux Toolkit split: part 1 by Vrushay (done), part 2 and globleState.js by Subhash (in progress).</t>
   </si>
   <si>
     <t xml:space="preserve">Design, Implementation</t>
   </si>
   <si>
+    <t xml:space="preserve">In progress</t>
+  </si>
+  <si>
     <t xml:space="preserve">11645a2, dbcae3a, 7ab1196 to 9809d35</t>
   </si>
   <si>
     <t xml:space="preserve">Super Admin and onboarding</t>
   </si>
   <si>
-    <t xml:space="preserve">Subhash, Vrushay, Tanya (onboarding)</t>
+    <t xml:space="preserve">Vrushay (Super Admin), Tanya (onboarding)</t>
   </si>
   <si>
     <t xml:space="preserve">Super Admin pages: dashboard, stores, store details, pending requests, subscription plans, settings. Login, forgot password and onboarding.</t>
@@ -106,7 +109,7 @@
     <t xml:space="preserve">Implementation</t>
   </si>
   <si>
-    <t xml:space="preserve">7307504 (onboarding owner details)</t>
+    <t xml:space="preserve">26 Super Admin commits, 7307504 (onboarding owner details)</t>
   </si>
   <si>
     <t xml:space="preserve">Store module</t>
@@ -139,9 +142,6 @@
     <t xml:space="preserve">Postman report and 96-case sheet done. Run the collection with all role tokens, record results, negative and security tests, bug fixes.</t>
   </si>
   <si>
-    <t xml:space="preserve">In progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">9e2ca1a, 8172cb7 (report), test case sheet</t>
   </si>
   <si>
@@ -211,13 +211,13 @@
     <t xml:space="preserve">bohra0022</t>
   </si>
   <si>
-    <t xml:space="preserve">Redux Toolkit part 1, frontend setup, Super Admin (with Subhash)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 Redux features, API client, utils</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dbcae3a, 7ab1196, 0abb5fc, 06b282a, 09a4708, 26e7b01, 8d7cd95, b04b449, ed775da, e426064, c579b5a, 9809d35</t>
+    <t xml:space="preserve">Redux Toolkit part 1, frontend setup, Super Admin, routing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 Redux features, API client, utils, 6 Super Admin pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45 frontend commits: Super Admin 26, Redux Toolkit 12, Setup 6, Routing 1</t>
   </si>
   <si>
     <t xml:space="preserve">Subhash Dhaka</t>
@@ -226,189 +226,231 @@
     <t xml:space="preserve">subhash8729</t>
   </si>
   <si>
-    <t xml:space="preserve">Folder structure, Redux Toolkit part 2, Super Admin (with Vrushay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 Super Admin pages; Redux: payment, product, refund, sale, shiftReport, store, storeAnalytics, subscription, subscriptionPlan, transaction, user, globleState.js</t>
+    <t xml:space="preserve">Folder structure, Redux Toolkit part 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux: payment, product, refund, sale, shiftReport, store, storeAnalytics, subscription, subscriptionPlan, transaction, user, globleState.js</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 frontend commits: Redux Toolkit 1, Setup 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vimal Kumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iamvkb7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 pages: create order, orders, returns, customers, shift summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40 frontend commits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishvas Choubisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choubisavishvas-web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 pages: dashboard, orders, refunds, transactions, inventory, employees, customers, reports, settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35 frontend commits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanya Singh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tanyasingh077</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store (largest module) and onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 pages: dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 frontend commits: Store 8, Auth and onboarding 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total pages across modules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend commits by member and module (from Git, 10 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend commits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux Toolkit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup and shared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Routing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auth and onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run reports/04-weekly-progress/make_commit_log.py for the latest numbers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work completed so far</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team repo and report folders set up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly Progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80c721c, 4584088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full Spring Boot backend uploaded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ef6144e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project idea, abstract and objectives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea &amp; Abstract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">see commit_log.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Features, modules and tech stack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS / Documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13dc390</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend folder structure (Subhash)</t>
   </si>
   <si>
     <t xml:space="preserve">ddf392b, 751e82d</t>
   </si>
   <si>
-    <t xml:space="preserve">Vimal Kumar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iamvkb7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cashier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 pages: create order, orders, returns, customers, shift summary</t>
+    <t xml:space="preserve">Frontend config, API client and utils (Vrushay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dbcae3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux Toolkit part 1, 11 features (Vrushay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7ab1196 to 9809d35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit log updates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">046f470, 67e0b4c, 8360f7e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UML, ER and architecture diagrams (20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11645a2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postman testing report, 2 parts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9e2ca1a, 8172cb7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">README with weekly plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b0ebffe, cdd3a24, b4bee2d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-week timeline and tracker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75398a4, 28069ac, 65daf38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week 1 report and weekly template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4430a3c, 7ce4830</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API test case sheet (96 cases)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POS_Backend_Test_Cases.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Made, not committed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager module (Vishvas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3197520, bb95311, db9c60b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier module (Vimal)</t>
   </si>
   <si>
     <t xml:space="preserve">3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
   </si>
   <si>
-    <t xml:space="preserve">Vishvas Choubisa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">choubisavishvas-web</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 pages: dashboard, orders, refunds, transactions, inventory, employees, customers, reports, settings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3197520, bb95311, db9c60b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tanya Singh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tanyasingh077</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store (largest module) and onboarding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 pages: dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts</t>
+    <t xml:space="preserve">Store module and onboarding (Tanya)</t>
   </si>
   <si>
     <t xml:space="preserve">7307504</t>
   </si>
   <si>
-    <t xml:space="preserve">Total pages across modules</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run reports/04-weekly-progress/make_commit_log.py to get exact commit counts per member and module.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work completed so far</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Team repo and report folders set up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80c721c, 4584088</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full Spring Boot backend uploaded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ef6144e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project idea, abstract and objectives</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idea &amp; Abstract</t>
-  </si>
-  <si>
-    <t xml:space="preserve">see commit_log.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Features, modules and tech stack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS / Documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13dc390</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend folder structure (Subhash)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend config, API client and utils (Vrushay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dbcae3a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redux Toolkit part 1, 11 features (Vrushay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7ab1196 to 9809d35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commit log updates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">046f470, 67e0b4c, 8360f7e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UML, ER and architecture diagrams (20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11645a2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postman testing report, 2 parts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9e2ca1a, 8172cb7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">README with weekly plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b0ebffe, cdd3a24, b4bee2d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10-week timeline and tracker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">75398a4, 28069ac, 65daf38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 1 report and weekly template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4430a3c, 7ce4830</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API test case sheet (96 cases)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POS_Backend_Test_Cases.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Made, not committed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager module (Vishvas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cashier module (Vimal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store module and onboarding (Tanya)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin module (Subhash and Vrushay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">commits in the team repo</t>
+    <t xml:space="preserve">Super Admin module (Vrushay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 commits, see frontend_work_log.csv</t>
   </si>
   <si>
     <t xml:space="preserve">Redux Toolkit part 2 and globleState.js (Subhash)</t>
   </si>
   <si>
+    <t xml:space="preserve">1 commit so far</t>
+  </si>
+  <si>
     <t xml:space="preserve">Run the Postman collection and record results</t>
   </si>
   <si>
@@ -454,7 +496,7 @@
     <t xml:space="preserve">Commit log, frontend work log, timeline and weekly reports. Update every week.</t>
   </si>
   <si>
-    <t xml:space="preserve">Backend, Redux Toolkit and all frontend modules done. Code quality fixes pending.</t>
+    <t xml:space="preserve">Backend and four frontend modules done. Redux part 2 and code quality fixes pending.</t>
   </si>
   <si>
     <t xml:space="preserve">Report and 96 test cases written, results to be recorded.</t>
@@ -1051,10 +1093,10 @@
         <v>21</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1070,22 +1112,22 @@
         <v>46229</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>16</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1101,16 +1143,16 @@
         <v>46236</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>16</v>
@@ -1130,22 +1172,22 @@
         <v>46243</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>16</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1161,19 +1203,19 @@
         <v>46250</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E11" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>35</v>
-      </c>
       <c r="H11" s="11" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>39</v>
@@ -1201,7 +1243,7 @@
         <v>42</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>43</v>
@@ -1301,16 +1343,16 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"Done")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"In progress")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1344,7 +1386,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -1399,7 +1441,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>65</v>
       </c>
@@ -1416,7 +1458,7 @@
         <v>69</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1488,9 +1530,144 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
         <v>86</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <f aca="false">SUM(C14:C23)</f>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1522,15 +1699,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>9</v>
@@ -1550,16 +1727,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>16</v>
@@ -1570,16 +1747,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>16</v>
@@ -1590,16 +1767,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>16</v>
@@ -1610,16 +1787,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>16</v>
@@ -1630,16 +1807,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>69</v>
+        <v>111</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>16</v>
@@ -1650,16 +1827,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>16</v>
@@ -1670,16 +1847,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>16</v>
@@ -1690,16 +1867,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>16</v>
@@ -1710,16 +1887,16 @@
         <v>9</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>16</v>
@@ -1730,16 +1907,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>16</v>
@@ -1750,16 +1927,16 @@
         <v>11</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>16</v>
@@ -1770,16 +1947,16 @@
         <v>12</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>16</v>
@@ -1790,16 +1967,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>16</v>
@@ -1810,19 +1987,19 @@
         <v>14</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,16 +2007,16 @@
         <v>15</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>5</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>79</v>
+        <v>133</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>16</v>
@@ -1850,16 +2027,16 @@
         <v>16</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>5</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>74</v>
+        <v>135</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>16</v>
@@ -1870,16 +2047,16 @@
         <v>17</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D20" s="6" t="n">
         <v>4</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>84</v>
+        <v>137</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>16</v>
@@ -1890,16 +2067,16 @@
         <v>18</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>3</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>16</v>
@@ -1910,19 +2087,19 @@
         <v>19</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D22" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1930,19 +2107,19 @@
         <v>20</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1951,12 +2128,12 @@
       </c>
       <c r="C25" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"Done")</f>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="C26" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"Made, not committed")</f>
@@ -1965,16 +2142,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"In progress")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"Pending")</f>
@@ -2008,26 +2185,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>5</v>
@@ -2036,26 +2213,26 @@
         <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>10</v>
@@ -2064,21 +2241,21 @@
         <v>16</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>25</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2089,53 +2266,53 @@
         <v>20</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>10</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="D10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="D11" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">SUM(B4:B11)</f>
@@ -2144,7 +2321,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">SUMIF(C4:C11,"&lt;&gt;Not started",B4:B11)</f>
@@ -2153,7 +2330,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">B14/B13</f>

</xml_diff>

<commit_message>
docs(timeline): mark weeks 1 to 5 done and add the new assignment week
</commit_message>
<xml_diff>
--- a/reports/09-timeline/Project_Timeline.xlsx
+++ b/reports/09-timeline/Project_Timeline.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="165">
   <si>
     <t xml:space="preserve">POS System: 10-week project timeline</t>
   </si>
@@ -79,424 +79,427 @@
     <t xml:space="preserve">13dc390, 4584088, 80c721c, ef6144e, ddf392b, 751e82d</t>
   </si>
   <si>
-    <t xml:space="preserve">Design and Redux split</t>
+    <t xml:space="preserve">Design and Redux Toolkit</t>
   </si>
   <si>
     <t xml:space="preserve">Vrushay, Subhash</t>
   </si>
   <si>
-    <t xml:space="preserve">UML and ER diagrams (done), Redux Toolkit split: part 1 by Vrushay (done), part 2 and globleState.js by Subhash (in progress).</t>
+    <t xml:space="preserve">UML and ER diagrams, and Redux Toolkit fully done: part 1 by Vrushay, part 2 and globleState.js by Subhash.</t>
   </si>
   <si>
     <t xml:space="preserve">Design, Implementation</t>
   </si>
   <si>
+    <t xml:space="preserve">11645a2, dbcae3a, 7ab1196 to 9809d35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin and onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vrushay (Super Admin), Tanya (onboarding)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin pages: dashboard, stores, store details, pending requests, subscription plans, settings. Login, forgot password and onboarding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 Super Admin commits, 7307504 (onboarding owner details)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store pages (11): dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager and Cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishvas (Branch Manager), Vimal (Cashier)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager pages (9) and Cashier pages (5): POS screen, returns, order history, customer lookup, shift summary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3197520, bb95311, db9c60b, 3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vrushay with the whole team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postman report and 96-case sheet done. Run the collection with all role tokens, record results, negative and security tests, bug fixes.</t>
+  </si>
+  <si>
     <t xml:space="preserve">In progress</t>
   </si>
   <si>
-    <t xml:space="preserve">11645a2, dbcae3a, 7ab1196 to 9809d35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin and onboarding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vrushay (Super Admin), Tanya (onboarding)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin pages: dashboard, stores, store details, pending requests, subscription plans, settings. Login, forgot password and onboarding.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 Super Admin commits, 7307504 (onboarding owner details)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tanya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store pages (11): dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager and Cashier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vishvas (Branch Manager), Vimal (Cashier)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager pages (9) and Cashier pages (5): POS screen, returns, order history, customer lookup, shift summary.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3197520, bb95311, db9c60b, 3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vrushay with the whole team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postman report and 96-case sheet done. Run the collection with all role tokens, record results, negative and security tests, bug fixes.</t>
-  </si>
-  <si>
     <t xml:space="preserve">9e2ca1a, 8172cb7 (report), test case sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Payments and integration</t>
+    <t xml:space="preserve">New assignment (coming soon)</t>
   </si>
   <si>
     <t xml:space="preserve">Team</t>
   </si>
   <si>
-    <t xml:space="preserve">Razorpay and Stripe checkout, subscription upgrade, payment status, email receipts, API integration.</t>
+    <t xml:space="preserve">New assignment to be announced. This week will be updated once it is known.</t>
   </si>
   <si>
     <t xml:space="preserve">Planned</t>
   </si>
   <si>
-    <t xml:space="preserve">Code quality, SRS and documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS in IEEE format, Axios interceptor, logout fix, API URL in env file, remove console logs, fix security findings, update README.</t>
+    <t xml:space="preserve">Payments, SRS and documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Razorpay and Stripe checkout, subscription upgrade, SRS in IEEE format, Axios interceptor, logout fix, API URL in env file, remove console logs, update README.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS / Documentation, Implementation &amp; Code Quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentation and viva prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report PPT, demo script, viva questions, final documents.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentation, Demo &amp; Viva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final demo and submission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full demo run, final checks, final commit log, submission.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo &amp; Viva, Weekly Progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend work log: who built which module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Known commits (to 10 Oct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vrushay Bohra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bohra0022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux Toolkit part 1, frontend setup, Super Admin, routing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 Redux features, API client, utils, 6 Super Admin pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45 frontend commits: Super Admin 26, Redux Toolkit 12, Setup 6, Routing 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subhash Dhaka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">subhash8729</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folder structure, Redux Toolkit part 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux: payment, product, refund, sale, shiftReport, store, storeAnalytics, subscription, subscriptionPlan, transaction, user, globleState.js</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux part 2 and globleState.js pushed after the 10 Oct count. Re-run make_commit_log.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vimal Kumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iamvkb7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 pages: create order, orders, returns, customers, shift summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40 frontend commits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishvas Choubisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choubisavishvas-web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 pages: dashboard, orders, refunds, transactions, inventory, employees, customers, reports, settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35 frontend commits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanya Singh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tanyasingh077</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store (largest module) and onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 pages: dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 frontend commits: Store 8, Auth and onboarding 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total pages across modules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend commits by member and module (from Git, 10 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend commits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux Toolkit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup and shared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Routing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auth and onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run reports/04-weekly-progress/make_commit_log.py for the latest numbers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work completed so far</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team repo and report folders set up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly Progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80c721c, 4584088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full Spring Boot backend uploaded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ef6144e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project idea, abstract and objectives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea &amp; Abstract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">see commit_log.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Features, modules and tech stack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS / Documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13dc390</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend folder structure (Subhash)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ddf392b, 751e82d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend config, API client and utils (Vrushay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dbcae3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux Toolkit part 1, 11 features (Vrushay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7ab1196 to 9809d35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit log updates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">046f470, 67e0b4c, 8360f7e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UML, ER and architecture diagrams (20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11645a2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postman testing report, 2 parts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9e2ca1a, 8172cb7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">README with weekly plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b0ebffe, cdd3a24, b4bee2d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-week timeline and tracker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75398a4, 28069ac, 65daf38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week 1 report and weekly template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4430a3c, 7ce4830</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API test case sheet (96 cases)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POS_Backend_Test_Cases.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Made, not committed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager module (Vishvas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3197520, bb95311, db9c60b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier module (Vimal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store module and onboarding (Tanya)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7307504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Admin module (Vrushay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 commits, see frontend_work_log.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redux Toolkit part 2 and globleState.js (Subhash)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">see frontend_work_log.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run the Postman collection and record results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test case sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Progress by marks component</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Component</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Committed in reports.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IEEE format SRS still to be written.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design (Use-case, Class, ER)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 diagrams committed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly Progress (tracking sheet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit log, frontend work log, timeline and weekly reports. Update every week.</t>
   </si>
   <si>
     <t xml:space="preserve">Implementation &amp; Code Quality</t>
   </si>
   <si>
-    <t xml:space="preserve">Presentation and viva prep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Report PPT, demo script, viva questions, final documents.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presentation, Demo &amp; Viva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Final demo and submission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full demo run, final checks, final commit log, submission.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demo &amp; Viva, Weekly Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done weeks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend work log: who built which module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Member</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GitHub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Known commits (to 10 Oct)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vrushay Bohra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bohra0022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redux Toolkit part 1, frontend setup, Super Admin, routing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 Redux features, API client, utils, 6 Super Admin pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45 frontend commits: Super Admin 26, Redux Toolkit 12, Setup 6, Routing 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subhash Dhaka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">subhash8729</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Folder structure, Redux Toolkit part 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redux: payment, product, refund, sale, shiftReport, store, storeAnalytics, subscription, subscriptionPlan, transaction, user, globleState.js</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 frontend commits: Redux Toolkit 1, Setup 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vimal Kumar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iamvkb7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cashier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 pages: create order, orders, returns, customers, shift summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40 frontend commits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vishvas Choubisa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">choubisavishvas-web</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 pages: dashboard, orders, refunds, transactions, inventory, employees, customers, reports, settings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35 frontend commits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tanya Singh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tanyasingh077</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store (largest module) and onboarding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 pages: dashboard, branches, categories, employees, products, stores, sales, reports, upgrade, settings, alerts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 frontend commits: Store 8, Auth and onboarding 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total pages across modules</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend commits by member and module (from Git, 10 Oct 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend commits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redux Toolkit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Setup and shared</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Routing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auth and onboarding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run reports/04-weekly-progress/make_commit_log.py for the latest numbers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work completed so far</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Team repo and report folders set up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80c721c, 4584088</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full Spring Boot backend uploaded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ef6144e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project idea, abstract and objectives</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idea &amp; Abstract</t>
-  </si>
-  <si>
-    <t xml:space="preserve">see commit_log.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Features, modules and tech stack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS / Documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13dc390</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend folder structure (Subhash)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ddf392b, 751e82d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frontend config, API client and utils (Vrushay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dbcae3a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redux Toolkit part 1, 11 features (Vrushay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7ab1196 to 9809d35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commit log updates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">046f470, 67e0b4c, 8360f7e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UML, ER and architecture diagrams (20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11645a2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postman testing report, 2 parts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9e2ca1a, 8172cb7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">README with weekly plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b0ebffe, cdd3a24, b4bee2d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10-week timeline and tracker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">75398a4, 28069ac, 65daf38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Week 1 report and weekly template</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4430a3c, 7ce4830</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API test case sheet (96 cases)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POS_Backend_Test_Cases.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Made, not committed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager module (Vishvas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3197520, bb95311, db9c60b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cashier module (Vimal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store module and onboarding (Tanya)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7307504</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Admin module (Vrushay)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 commits, see frontend_work_log.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redux Toolkit part 2 and globleState.js (Subhash)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 commit so far</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run the Postman collection and record results</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test case sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Progress by marks component</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Component</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Committed in reports.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IEEE format SRS still to be written.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design (Use-case, Class, ER)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 diagrams committed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly Progress (tracking sheet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commit log, frontend work log, timeline and weekly reports. Update every week.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backend and four frontend modules done. Redux part 2 and code quality fixes pending.</t>
+    <t xml:space="preserve">Backend, Redux Toolkit (22 features) and four frontend modules done. Code quality fixes pending.</t>
   </si>
   <si>
     <t xml:space="preserve">Report and 96 test cases written, results to be recorded.</t>
@@ -1093,10 +1096,10 @@
         <v>21</v>
       </c>
       <c r="H7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1112,22 +1115,22 @@
         <v>46229</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,16 +1146,16 @@
         <v>46236</v>
       </c>
       <c r="D9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>31</v>
-      </c>
       <c r="G9" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>16</v>
@@ -1172,22 +1175,22 @@
         <v>46243</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1203,25 +1206,25 @@
         <v>46250</v>
       </c>
       <c r="D11" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>22</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
         <v>7</v>
       </c>
@@ -1243,14 +1246,14 @@
         <v>42</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>43</v>
       </c>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="n">
         <v>8</v>
       </c>
@@ -1343,16 +1346,16 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"Done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"In progress")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1458,7 +1461,7 @@
         <v>69</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1750,7 +1753,7 @@
         <v>102</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>1</v>
@@ -1810,7 +1813,7 @@
         <v>110</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>1</v>
@@ -1830,7 +1833,7 @@
         <v>112</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>2</v>
@@ -1850,7 +1853,7 @@
         <v>114</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>2</v>
@@ -1910,7 +1913,7 @@
         <v>121</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>6</v>
@@ -1990,7 +1993,7 @@
         <v>129</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>6</v>
@@ -2010,7 +2013,7 @@
         <v>132</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>5</v>
@@ -2030,7 +2033,7 @@
         <v>134</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>5</v>
@@ -2050,7 +2053,7 @@
         <v>136</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20" s="6" t="n">
         <v>4</v>
@@ -2070,7 +2073,7 @@
         <v>138</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>3</v>
@@ -2090,7 +2093,7 @@
         <v>140</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D22" s="6" t="n">
         <v>2</v>
@@ -2099,7 +2102,7 @@
         <v>141</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,7 +2113,7 @@
         <v>142</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>6</v>
@@ -2119,7 +2122,7 @@
         <v>143</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2128,7 +2131,7 @@
       </c>
       <c r="C25" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"Done")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2142,11 +2145,11 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">COUNTIF(F4:F23,"In progress")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2260,7 +2263,7 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>46</v>
+        <v>157</v>
       </c>
       <c r="B8" s="6" t="n">
         <v>20</v>
@@ -2269,12 +2272,12 @@
         <v>155</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>10</v>
@@ -2283,12 +2286,12 @@
         <v>155</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>10</v>
@@ -2300,7 +2303,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>10</v>
@@ -2312,7 +2315,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">SUM(B4:B11)</f>
@@ -2321,7 +2324,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">SUMIF(C4:C11,"&lt;&gt;Not started",B4:B11)</f>
@@ -2330,7 +2333,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">B14/B13</f>

</xml_diff>

<commit_message>
docs(timeline): mark all weeks done
</commit_message>
<xml_diff>
--- a/reports/09-timeline/Project_Timeline.xlsx
+++ b/reports/09-timeline/Project_Timeline.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="177">
   <si>
     <t xml:space="preserve">POS System: 10-week project timeline</t>
   </si>
@@ -136,57 +136,69 @@
     <t xml:space="preserve">Vrushay with the whole team</t>
   </si>
   <si>
-    <t xml:space="preserve">Postman report and 96-case sheet done. Run the collection with all role tokens, record results, negative and security tests, bug fixes.</t>
+    <t xml:space="preserve">Postman API testing report in two parts and a sheet of 96 test cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/06-testing/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payments and integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Razorpay and Stripe payment services, subscription flows, and the payment, subscription and subscription plan Redux features.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend payment module, Redux features</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS and documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requirements specification (SRS) and POS system documentation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS / Documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/02-srs/, reports/05-implementation/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentation and viva prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report presentation and viva questions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentation, Demo &amp; Viva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/07-presentation/, reports/08-demo-viva/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final report and submission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project report, final commit logs and submission.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly Progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/10-project-report/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done weeks</t>
   </si>
   <si>
     <t xml:space="preserve">In progress</t>
   </si>
   <si>
-    <t xml:space="preserve">9e2ca1a, 8172cb7 (report), test case sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New assignment (coming soon)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New assignment to be announced. This week will be updated once it is known.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Planned</t>
   </si>
   <si>
-    <t xml:space="preserve">Payments, SRS and documentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Razorpay and Stripe checkout, subscription upgrade, SRS in IEEE format, Axios interceptor, logout fix, API URL in env file, remove console logs, update README.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRS / Documentation, Implementation &amp; Code Quality</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presentation and viva prep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Report PPT, demo script, viva questions, final documents.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presentation, Demo &amp; Viva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Final demo and submission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full demo run, final checks, final commit log, submission.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demo &amp; Viva, Weekly Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done weeks</t>
-  </si>
-  <si>
     <t xml:space="preserve">Frontend work log: who built which module</t>
   </si>
   <si>
@@ -325,9 +337,6 @@
     <t xml:space="preserve">Team repo and report folders set up</t>
   </si>
   <si>
-    <t xml:space="preserve">Weekly Progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">80c721c, 4584088</t>
   </si>
   <si>
@@ -349,9 +358,6 @@
     <t xml:space="preserve">Features, modules and tech stack</t>
   </si>
   <si>
-    <t xml:space="preserve">SRS / Documentation</t>
-  </si>
-  <si>
     <t xml:space="preserve">13dc390</t>
   </si>
   <si>
@@ -451,10 +457,40 @@
     <t xml:space="preserve">see frontend_work_log.csv</t>
   </si>
   <si>
-    <t xml:space="preserve">Run the Postman collection and record results</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test case sheet</t>
+    <t xml:space="preserve">Requirements specification (SRS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/02-srs/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POS system documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/05-implementation/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/07-presentation/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viva questions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo &amp; Viva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reports/08-demo-viva/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run the Postman collection and record results in the test sheet</t>
   </si>
   <si>
     <t xml:space="preserve">Pending</t>
@@ -475,10 +511,7 @@
     <t xml:space="preserve">Committed in reports.</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IEEE format SRS still to be written.</t>
+    <t xml:space="preserve">SRS and documentation are in reports.</t>
   </si>
   <si>
     <t xml:space="preserve">Design (Use-case, Class, ER)</t>
@@ -505,10 +538,13 @@
     <t xml:space="preserve">Report and 96 test cases written, results to be recorded.</t>
   </si>
   <si>
-    <t xml:space="preserve">Presentation</t>
+    <t xml:space="preserve">Report presentation is in reports.</t>
   </si>
   <si>
     <t xml:space="preserve">Demo &amp; Viva (individual)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viva questions written. Demo still to present.</t>
   </si>
   <si>
     <t xml:space="preserve">Total marks</t>
@@ -1193,7 +1229,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="n">
         <v>6</v>
       </c>
@@ -1218,13 +1254,13 @@
         <v>35</v>
       </c>
       <c r="H11" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I11" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
         <v>7</v>
       </c>
@@ -1237,23 +1273,25 @@
         <v>46257</v>
       </c>
       <c r="D12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>42</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="I12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="n">
         <v>8</v>
       </c>
@@ -1266,21 +1304,23 @@
         <v>46264</v>
       </c>
       <c r="D13" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="9" t="s">
+      <c r="G13" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="H13" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H13" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
@@ -1298,7 +1338,7 @@
         <v>47</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>48</v>
@@ -1307,9 +1347,11 @@
         <v>49</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="I14" s="6"/>
+        <v>16</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="n">
@@ -1324,47 +1366,49 @@
         <v>46278</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I15" s="9"/>
+        <v>16</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"Done")</f>
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"In progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">COUNTIF(H6:H15,"Planned")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1401,24 +1445,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>10</v>
@@ -1426,19 +1470,19 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>16</v>
@@ -1446,19 +1490,19 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>16</v>
@@ -1466,19 +1510,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>16</v>
@@ -1486,19 +1530,19 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>16</v>
@@ -1506,19 +1550,19 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>16</v>
@@ -1526,7 +1570,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D10" s="12" t="n">
         <f aca="false">6+5+9+11</f>
@@ -1535,26 +1579,26 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C14" s="8" t="n">
         <v>26</v>
@@ -1562,10 +1606,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C15" s="11" t="n">
         <v>12</v>
@@ -1573,10 +1617,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>6</v>
@@ -1584,10 +1628,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C17" s="11" t="n">
         <v>1</v>
@@ -1595,10 +1639,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>40</v>
@@ -1606,10 +1650,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C19" s="11" t="n">
         <v>35</v>
@@ -1617,10 +1661,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>8</v>
@@ -1628,10 +1672,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C21" s="11" t="n">
         <v>3</v>
@@ -1639,10 +1683,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>2</v>
@@ -1650,10 +1694,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C23" s="11" t="n">
         <v>1</v>
@@ -1661,7 +1705,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C24" s="2" t="n">
         <f aca="false">SUM(C14:C23)</f>
@@ -1670,7 +1714,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1689,7 +1733,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1702,15 +1746,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>9</v>
@@ -1730,16 +1774,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>16</v>
@@ -1750,7 +1794,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>26</v>
@@ -1759,7 +1803,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>16</v>
@@ -1770,16 +1814,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>16</v>
@@ -1790,16 +1834,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>16</v>
@@ -1810,7 +1854,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>26</v>
@@ -1819,7 +1863,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>16</v>
@@ -1830,7 +1874,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>26</v>
@@ -1839,7 +1883,7 @@
         <v>2</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>16</v>
@@ -1850,7 +1894,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>26</v>
@@ -1859,7 +1903,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>16</v>
@@ -1870,16 +1914,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>16</v>
@@ -1890,16 +1934,16 @@
         <v>9</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>16</v>
@@ -1910,7 +1954,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>35</v>
@@ -1919,7 +1963,7 @@
         <v>6</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>16</v>
@@ -1930,16 +1974,16 @@
         <v>11</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>16</v>
@@ -1950,16 +1994,16 @@
         <v>12</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>16</v>
@@ -1970,16 +2014,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>16</v>
@@ -1990,7 +2034,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>35</v>
@@ -1999,10 +2043,10 @@
         <v>6</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2010,7 +2054,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>26</v>
@@ -2019,7 +2063,7 @@
         <v>5</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>16</v>
@@ -2030,7 +2074,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>26</v>
@@ -2039,7 +2083,7 @@
         <v>5</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>16</v>
@@ -2050,7 +2094,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>26</v>
@@ -2059,7 +2103,7 @@
         <v>4</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>16</v>
@@ -2070,7 +2114,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>26</v>
@@ -2079,7 +2123,7 @@
         <v>3</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>16</v>
@@ -2090,7 +2134,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>26</v>
@@ -2099,7 +2143,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>16</v>
@@ -2110,54 +2154,154 @@
         <v>20</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D28" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E23" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="12" t="n">
-        <f aca="false">COUNTIF(F4:F23,"Done")</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C26" s="12" t="n">
-        <f aca="false">COUNTIF(F4:F23,"Made, not committed")</f>
+      <c r="E28" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="12" t="n">
+        <f aca="false">COUNTIF(F4:F28,"Done")</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C31" s="12" t="n">
+        <f aca="false">COUNTIF(F4:F28,"Made, not committed")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C27" s="12" t="n">
-        <f aca="false">COUNTIF(F4:F23,"In progress")</f>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="12" t="n">
+        <f aca="false">COUNTIF(F4:F28,"In progress")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C28" s="12" t="n">
-        <f aca="false">COUNTIF(F4:F23,"Pending")</f>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <f aca="false">COUNTIF(F4:F28,"Pending")</f>
         <v>0</v>
       </c>
     </row>
@@ -2188,26 +2332,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>5</v>
@@ -2216,26 +2360,26 @@
         <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>150</v>
+        <v>16</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>10</v>
@@ -2244,35 +2388,35 @@
         <v>16</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>25</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="B8" s="6" t="n">
         <v>20</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2283,39 +2427,43 @@
         <v>10</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>10</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="D10" s="6"/>
+        <v>16</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="D11" s="9"/>
+        <v>166</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">SUM(B4:B11)</f>
@@ -2324,20 +2472,20 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">SUMIF(C4:C11,"&lt;&gt;Not started",B4:B11)</f>
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">B14/B13</f>
-        <v>0.7</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>